<commit_message>
Fix monitoring: SSL bypass, timeout 30s, wider keywords, sources update
monitor.py:
- Add urllib3.disable_warnings for sites with self-signed certs (voda.gov.ru)
- Increase request timeout 20s → 30s, add verify=False
- Expand INCLUDE_KEYWORDS: add word stems (земл, лесн, недвижимост,
  экологич, аренд, природн, регистраци, оформлени), broader terms for
  real estate, ecology, nature protection — reduces false negatives

sources.xlsx:
- Fix Garant URL: /actual/zemlya/ (404) → /news/ (working)
- Add Картотека арб. дел (kad.arbitr.ru)
- Add Правовые акты России (pravo.gov.ru)
- Total active sources: 7 (was 5)

https://claude.ai/code/session_01JfZnWsmLGa67xbmvY4GjdU
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -437,11 +437,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -537,12 +537,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Гарант — земельное право</t>
+          <t>Гарант — новости законодательства</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://www.garant.ru/actual/zemlya/</t>
+          <t>https://www.garant.ru/news/</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -559,7 +559,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>КонсультантПлюс — новости законодательства</t>
+          <t>КонсультантПлюс — новости</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -581,42 +581,86 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Росводресурсы (TG)</t>
+          <t>Картотека арб. дел (КАД)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/rosvod_ru</t>
+          <t>https://kad.arbitr.ru/</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>telegram</t>
+          <t>site</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>нет</t>
+          <t>да</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Правовые акты России</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>https://pravo.gov.ru/proxy/ips/?start_search&amp;fattribs=true</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Росводресурсы (TG)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/rosvod_ru</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Росреестр (TG)</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>https://t.me/rosreestr_official</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>telegram</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>нет</t>
         </is>

</xml_diff>

<commit_message>
Update sources.xlsx: 38 telegram + 13 site sources
Telegram (active=да, pending Telethon setup):
  vashecolog, yuristypronedvizhimost, minprirody, minleshoz,
  rosreestrnews, rosvodresursy, rosnedraofficial, zemelnoepravo,
  kadastr1, vodarossii, prozemli, zemadvokat, природа and 25 more

Sites (active=да, parsed via BeautifulSoup):
  Росреестр, Росводресурсы, Рослесхоз, Минприроды, Гарант,
  КонсультантПлюс, pravo.ru, pravoved.ru, Адвокатская газета,
  КАД Арбитр, sudrf.ru, vodnkod.ru, profcadastre.ru

https://claude.ai/code/session_01JfZnWsmLGa67xbmvY4GjdU
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -44,12 +44,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBF3FB"/>
+        <fgColor rgb="00E8F4FD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F8EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0F2DD"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,13 +75,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -437,11 +449,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -471,17 +483,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Росводресурсы</t>
+          <t>vashecolog</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>https://voda.gov.ru</t>
+          <t>https://t.me/vashecolog</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>telegram</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -493,17 +505,17 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Росреестр — пресс-архив</t>
+          <t>yuristypronedvizhimost</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://rosreestr.gov.ru/press/archive/</t>
+          <t>https://t.me/yuristypronedvizhimost</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>telegram</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -515,17 +527,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Минприроды России — новости</t>
+          <t>minprirody</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://www.mnr.gov.ru/press/news/</t>
+          <t>https://t.me/minprirody</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>telegram</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -537,17 +549,17 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Гарант — новости законодательства</t>
+          <t>minleshoz</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://www.garant.ru/news/</t>
+          <t>https://t.me/minleshoz</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>telegram</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -559,17 +571,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>КонсультантПлюс — новости</t>
+          <t>sroskisoyuz</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://www.consultant.ru/law/hotdocs/</t>
+          <t>https://t.me/sroskisoyuz</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>telegram</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -581,17 +593,17 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Картотека арб. дел (КАД)</t>
+          <t>nedvijka</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/</t>
+          <t>https://t.me/nedvijka</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>telegram</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -603,17 +615,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Правовые акты России</t>
+          <t>ekologiapravochat</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://pravo.gov.ru/proxy/ips/?start_search&amp;fattribs=true</t>
+          <t>https://t.me/ekologiapravochat</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>telegram</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -625,12 +637,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Росводресурсы (TG)</t>
+          <t>stroikiitochka</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>https://t.me/rosvod_ru</t>
+          <t>https://t.me/stroikiitochka</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -640,19 +652,19 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>нет</t>
+          <t>да</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Росреестр (TG)</t>
+          <t>bezdelkaBuh</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://t.me/rosreestr_official</t>
+          <t>https://t.me/bezdelkaBuh</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -662,7 +674,931 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>нет</t>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>zemelnyfond</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/zemelnyfond</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>zhelnintax</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/zhelnintax</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>zakonystroiki</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/zakonystroiki</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>kadastr1</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/kadastr1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>ecoeventru</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/ecoeventru</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Rosleshozofficial</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/Rosleshozofficial</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>rpngov</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/rpngov</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>dvizhenieru</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/dvizhenieru</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>rosreestrnews</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/rosreestrnews</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>rosimushchestvo</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/rosimushchestvo</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>rosvodresursy</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/rosvodresursy</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>prozemli</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/prozemli</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>zemelnoepravo</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/zemelnoepravo</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>consultantplus</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/consultantplus</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>stroinews</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/stroinews</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>rosnedraofficial</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/rosnedraofficial</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>zemelnyvopros</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/zemelnyvopros</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>zemelnyjfond</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/zemelnyjfond</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>ecotexpert</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/ecotexpert</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>uristpozemle</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/uristpozemle</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>bezdelkabuh</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/bezdelkabuh</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>uristvnedvijke</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/uristvnedvijke</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>vodarossii</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/vodarossii</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>tolstihinainvest</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/tolstihinainvest</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>nedvizhimostzakon</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/nedvizhimostzakon</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>erznews</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/erznews</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>minprirodyrf</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/minprirodyrf</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>zemadvokat</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>https://t.me/zemadvokat</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>priroda</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>https://t.me/prirodaru</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>telegram</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Росреестр</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>https://rosreestr.gov.ru</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Росводресурсы</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>https://voda.gov.ru</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Рослесхоз</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>https://rosleshoz.gov.ru</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Минприроды</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>https://mnr.gov.ru</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Гарант новости</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>https://www.garant.ru/news/</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>КонсультантПлюс</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>https://www.consultant.ru/law/hotdocs/</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>pravo.ru</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>https://pravo.ru</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>pravoved.ru</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>https://pravoved.ru</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Адвокатская газета</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>https://advgazeta.ru</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>КАД Арбитр</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>sudrf.ru</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>https://sudrf.ru</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>vodnkod.ru</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>https://vodnkod.ru</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>profcadastre.ru</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>https://profcadastre.ru</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>site</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>да</t>
         </is>
       </c>
     </row>

</xml_diff>